<commit_message>
mise à jour de pages
Ajout de liens et réécriture des textes
</commit_message>
<xml_diff>
--- a/Images/Tableau de synthèse - Debaisieux Matthieu.xlsx
+++ b/Images/Tableau de synthèse - Debaisieux Matthieu.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mrpio\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dbf579e00f6a4d0d/Desktop/Codage/Dossier pro/Images/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48AB5734-CBC2-4D0C-8D3C-F0EC87EAF822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{48AB5734-CBC2-4D0C-8D3C-F0EC87EAF822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{841F3384-67E0-4145-9660-0F08ED2725F1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,10 +201,10 @@
     <t>06/05/2026 au 02/09/2027</t>
   </si>
   <si>
-    <t>Création d'n site web capable d’analyser une URL fournie par un utilisateur afin de générer un rapport SEO simplifié, clair et pédagogique.</t>
-  </si>
-  <si>
     <t>13/07/2026 au 10/08/2026</t>
+  </si>
+  <si>
+    <t>Création d'un site web capable d’analyser une URL fournie par un utilisateur afin de générer un rapport SEO simplifié, clair et pédagogique.</t>
   </si>
 </sst>
 </file>
@@ -911,6 +911,15 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -991,15 +1000,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1327,27 +1327,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:59" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="59"/>
-      <c r="P1" s="59"/>
-      <c r="Q1" s="59"/>
-      <c r="R1" s="59"/>
-      <c r="S1" s="59"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="K1" s="62"/>
+      <c r="L1" s="62"/>
+      <c r="M1" s="62"/>
+      <c r="N1" s="62"/>
+      <c r="O1" s="62"/>
+      <c r="P1" s="62"/>
+      <c r="Q1" s="62"/>
+      <c r="R1" s="62"/>
+      <c r="S1" s="62"/>
       <c r="T1" s="17" t="s">
         <v>47</v>
       </c>
@@ -1385,142 +1385,142 @@
       <c r="X2" s="22"/>
     </row>
     <row r="3" spans="1:59" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="64" t="s">
+      <c r="A3" s="67" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="70"/>
-      <c r="C3" s="70"/>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
-      <c r="G3" s="70"/>
-      <c r="H3" s="70"/>
-      <c r="I3" s="70"/>
-      <c r="J3" s="70"/>
-      <c r="K3" s="70"/>
-      <c r="L3" s="70"/>
-      <c r="M3" s="70"/>
-      <c r="N3" s="70"/>
-      <c r="O3" s="70"/>
-      <c r="P3" s="70"/>
-      <c r="Q3" s="71"/>
-      <c r="R3" s="60" t="s">
+      <c r="B3" s="73"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="73"/>
+      <c r="J3" s="73"/>
+      <c r="K3" s="73"/>
+      <c r="L3" s="73"/>
+      <c r="M3" s="73"/>
+      <c r="N3" s="73"/>
+      <c r="O3" s="73"/>
+      <c r="P3" s="73"/>
+      <c r="Q3" s="74"/>
+      <c r="R3" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="S3" s="61"/>
-      <c r="T3" s="62"/>
-      <c r="U3" s="62"/>
-      <c r="V3" s="62"/>
-      <c r="W3" s="62"/>
-      <c r="X3" s="63"/>
+      <c r="S3" s="64"/>
+      <c r="T3" s="65"/>
+      <c r="U3" s="65"/>
+      <c r="V3" s="65"/>
+      <c r="W3" s="65"/>
+      <c r="X3" s="66"/>
     </row>
     <row r="4" spans="1:59" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="67" t="s">
+      <c r="A4" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="68"/>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
-      <c r="N4" s="68"/>
-      <c r="O4" s="68"/>
-      <c r="P4" s="68"/>
-      <c r="Q4" s="69"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="71"/>
+      <c r="H4" s="71"/>
+      <c r="I4" s="71"/>
+      <c r="J4" s="71"/>
+      <c r="K4" s="71"/>
+      <c r="L4" s="71"/>
+      <c r="M4" s="71"/>
+      <c r="N4" s="71"/>
+      <c r="O4" s="71"/>
+      <c r="P4" s="71"/>
+      <c r="Q4" s="72"/>
       <c r="R4" s="26"/>
       <c r="S4" s="23" t="s">
         <v>4</v>
       </c>
       <c r="T4" s="24"/>
-      <c r="U4" s="78" t="s">
+      <c r="U4" s="81" t="s">
         <v>45</v>
       </c>
-      <c r="V4" s="79"/>
+      <c r="V4" s="82"/>
       <c r="W4" s="25" t="s">
         <v>46</v>
       </c>
       <c r="X4" s="19"/>
     </row>
     <row r="5" spans="1:59" ht="40.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="64" t="s">
+      <c r="A5" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="65"/>
-      <c r="C5" s="65"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="65"/>
-      <c r="G5" s="65"/>
-      <c r="H5" s="65"/>
-      <c r="I5" s="65"/>
-      <c r="J5" s="65"/>
-      <c r="K5" s="65"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="65"/>
-      <c r="N5" s="65"/>
-      <c r="O5" s="65"/>
-      <c r="P5" s="65"/>
-      <c r="Q5" s="65"/>
-      <c r="R5" s="65"/>
-      <c r="S5" s="65"/>
-      <c r="T5" s="65"/>
-      <c r="U5" s="65"/>
-      <c r="V5" s="65"/>
-      <c r="W5" s="65"/>
-      <c r="X5" s="66"/>
+      <c r="B5" s="68"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="68"/>
+      <c r="F5" s="68"/>
+      <c r="G5" s="68"/>
+      <c r="H5" s="68"/>
+      <c r="I5" s="68"/>
+      <c r="J5" s="68"/>
+      <c r="K5" s="68"/>
+      <c r="L5" s="68"/>
+      <c r="M5" s="68"/>
+      <c r="N5" s="68"/>
+      <c r="O5" s="68"/>
+      <c r="P5" s="68"/>
+      <c r="Q5" s="68"/>
+      <c r="R5" s="68"/>
+      <c r="S5" s="68"/>
+      <c r="T5" s="68"/>
+      <c r="U5" s="68"/>
+      <c r="V5" s="68"/>
+      <c r="W5" s="68"/>
+      <c r="X5" s="69"/>
     </row>
     <row r="6" spans="1:59" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="83" t="s">
+      <c r="A6" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="84" t="s">
+      <c r="B6" s="87" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="75" t="s">
+      <c r="C6" s="78" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
-      <c r="F6" s="76"/>
-      <c r="G6" s="76"/>
-      <c r="H6" s="76"/>
-      <c r="I6" s="75" t="s">
+      <c r="D6" s="79"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="79"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
+      <c r="I6" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="J6" s="76"/>
-      <c r="K6" s="76"/>
-      <c r="L6" s="75" t="s">
+      <c r="J6" s="79"/>
+      <c r="K6" s="79"/>
+      <c r="L6" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="M6" s="76"/>
-      <c r="N6" s="76"/>
-      <c r="O6" s="75" t="s">
+      <c r="M6" s="79"/>
+      <c r="N6" s="79"/>
+      <c r="O6" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="P6" s="76"/>
-      <c r="Q6" s="76"/>
-      <c r="R6" s="75" t="s">
+      <c r="P6" s="79"/>
+      <c r="Q6" s="79"/>
+      <c r="R6" s="78" t="s">
         <v>12</v>
       </c>
-      <c r="S6" s="76"/>
-      <c r="T6" s="76"/>
-      <c r="U6" s="77" t="s">
+      <c r="S6" s="79"/>
+      <c r="T6" s="79"/>
+      <c r="U6" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="V6" s="77"/>
-      <c r="W6" s="77"/>
-      <c r="X6" s="77"/>
+      <c r="V6" s="80"/>
+      <c r="W6" s="80"/>
+      <c r="X6" s="80"/>
     </row>
     <row r="7" spans="1:59" s="2" customFormat="1" ht="390.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="83"/>
-      <c r="B7" s="84"/>
+      <c r="A7" s="86"/>
+      <c r="B7" s="87"/>
       <c r="C7" s="47" t="s">
         <v>14</v>
       </c>
@@ -1624,32 +1624,32 @@
       <c r="BG7" s="35"/>
     </row>
     <row r="8" spans="1:59" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="80" t="s">
+      <c r="A8" s="83" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="81"/>
-      <c r="C8" s="81"/>
-      <c r="D8" s="81"/>
-      <c r="E8" s="81"/>
-      <c r="F8" s="81"/>
-      <c r="G8" s="81"/>
-      <c r="H8" s="81"/>
-      <c r="I8" s="81"/>
-      <c r="J8" s="81"/>
-      <c r="K8" s="81"/>
-      <c r="L8" s="81"/>
-      <c r="M8" s="81"/>
-      <c r="N8" s="81"/>
-      <c r="O8" s="81"/>
-      <c r="P8" s="81"/>
-      <c r="Q8" s="81"/>
-      <c r="R8" s="81"/>
-      <c r="S8" s="81"/>
-      <c r="T8" s="81"/>
-      <c r="U8" s="81"/>
-      <c r="V8" s="81"/>
-      <c r="W8" s="81"/>
-      <c r="X8" s="82"/>
+      <c r="B8" s="84"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="84"/>
+      <c r="E8" s="84"/>
+      <c r="F8" s="84"/>
+      <c r="G8" s="84"/>
+      <c r="H8" s="84"/>
+      <c r="I8" s="84"/>
+      <c r="J8" s="84"/>
+      <c r="K8" s="84"/>
+      <c r="L8" s="84"/>
+      <c r="M8" s="84"/>
+      <c r="N8" s="84"/>
+      <c r="O8" s="84"/>
+      <c r="P8" s="84"/>
+      <c r="Q8" s="84"/>
+      <c r="R8" s="84"/>
+      <c r="S8" s="84"/>
+      <c r="T8" s="84"/>
+      <c r="U8" s="84"/>
+      <c r="V8" s="84"/>
+      <c r="W8" s="84"/>
+      <c r="X8" s="85"/>
       <c r="Y8"/>
       <c r="Z8"/>
       <c r="AA8"/>
@@ -2014,7 +2014,7 @@
     <row r="14" spans="1:59" s="2" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
       <c r="B14" s="54"/>
-      <c r="C14" s="85"/>
+      <c r="C14" s="58"/>
       <c r="D14" s="56"/>
       <c r="E14" s="56"/>
       <c r="F14" s="56"/>
@@ -2032,8 +2032,8 @@
       <c r="R14" s="56"/>
       <c r="S14" s="56"/>
       <c r="T14" s="56"/>
-      <c r="U14" s="86"/>
-      <c r="V14" s="87"/>
+      <c r="U14" s="59"/>
+      <c r="V14" s="60"/>
       <c r="W14" s="55"/>
       <c r="X14" s="56"/>
       <c r="Y14"/>
@@ -2317,32 +2317,32 @@
       <c r="BG18" s="35"/>
     </row>
     <row r="19" spans="1:59" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="72" t="s">
+      <c r="A19" s="75" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="73"/>
-      <c r="C19" s="73"/>
-      <c r="D19" s="73"/>
-      <c r="E19" s="73"/>
-      <c r="F19" s="73"/>
-      <c r="G19" s="73"/>
-      <c r="H19" s="73"/>
-      <c r="I19" s="73"/>
-      <c r="J19" s="73"/>
-      <c r="K19" s="73"/>
-      <c r="L19" s="73"/>
-      <c r="M19" s="73"/>
-      <c r="N19" s="73"/>
-      <c r="O19" s="73"/>
-      <c r="P19" s="73"/>
-      <c r="Q19" s="73"/>
-      <c r="R19" s="73"/>
-      <c r="S19" s="73"/>
-      <c r="T19" s="73"/>
-      <c r="U19" s="73"/>
-      <c r="V19" s="73"/>
-      <c r="W19" s="73"/>
-      <c r="X19" s="74"/>
+      <c r="B19" s="76"/>
+      <c r="C19" s="76"/>
+      <c r="D19" s="76"/>
+      <c r="E19" s="76"/>
+      <c r="F19" s="76"/>
+      <c r="G19" s="76"/>
+      <c r="H19" s="76"/>
+      <c r="I19" s="76"/>
+      <c r="J19" s="76"/>
+      <c r="K19" s="76"/>
+      <c r="L19" s="76"/>
+      <c r="M19" s="76"/>
+      <c r="N19" s="76"/>
+      <c r="O19" s="76"/>
+      <c r="P19" s="76"/>
+      <c r="Q19" s="76"/>
+      <c r="R19" s="76"/>
+      <c r="S19" s="76"/>
+      <c r="T19" s="76"/>
+      <c r="U19" s="76"/>
+      <c r="V19" s="76"/>
+      <c r="W19" s="76"/>
+      <c r="X19" s="77"/>
       <c r="Y19"/>
       <c r="Z19"/>
       <c r="AA19"/>
@@ -2381,10 +2381,10 @@
     </row>
     <row r="20" spans="1:59" s="2" customFormat="1" ht="38.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="54" t="s">
         <v>52</v>
-      </c>
-      <c r="B20" s="54" t="s">
-        <v>53</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="37"/>
@@ -2749,32 +2749,32 @@
       <c r="BG25" s="35"/>
     </row>
     <row r="26" spans="1:59" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A26" s="72" t="s">
+      <c r="A26" s="75" t="s">
         <v>43</v>
       </c>
-      <c r="B26" s="73"/>
-      <c r="C26" s="73"/>
-      <c r="D26" s="73"/>
-      <c r="E26" s="73"/>
-      <c r="F26" s="73"/>
-      <c r="G26" s="73"/>
-      <c r="H26" s="73"/>
-      <c r="I26" s="73"/>
-      <c r="J26" s="73"/>
-      <c r="K26" s="73"/>
-      <c r="L26" s="73"/>
-      <c r="M26" s="73"/>
-      <c r="N26" s="73"/>
-      <c r="O26" s="73"/>
-      <c r="P26" s="73"/>
-      <c r="Q26" s="73"/>
-      <c r="R26" s="73"/>
-      <c r="S26" s="73"/>
-      <c r="T26" s="73"/>
-      <c r="U26" s="73"/>
-      <c r="V26" s="73"/>
-      <c r="W26" s="73"/>
-      <c r="X26" s="74"/>
+      <c r="B26" s="76"/>
+      <c r="C26" s="76"/>
+      <c r="D26" s="76"/>
+      <c r="E26" s="76"/>
+      <c r="F26" s="76"/>
+      <c r="G26" s="76"/>
+      <c r="H26" s="76"/>
+      <c r="I26" s="76"/>
+      <c r="J26" s="76"/>
+      <c r="K26" s="76"/>
+      <c r="L26" s="76"/>
+      <c r="M26" s="76"/>
+      <c r="N26" s="76"/>
+      <c r="O26" s="76"/>
+      <c r="P26" s="76"/>
+      <c r="Q26" s="76"/>
+      <c r="R26" s="76"/>
+      <c r="S26" s="76"/>
+      <c r="T26" s="76"/>
+      <c r="U26" s="76"/>
+      <c r="V26" s="76"/>
+      <c r="W26" s="76"/>
+      <c r="X26" s="77"/>
       <c r="Y26"/>
       <c r="Z26"/>
       <c r="AA26"/>

</xml_diff>